<commit_message>
v1.1: corrected model inputs after source audit; add source dossier
- GREET phosphoric acid factor converted from short ton to tonne (1,379 kg CO2eq/t P2O5)
- FSA-route steam on the enthalpy basis of the steam price (14 GJ/t HF)
- Electronic-grade AHF input set to the disclosed design ratio (1.39)
- Capital-cost anchors and price ranges aligned with their sources
- Fig. A.1 US import unit value band corrected to 2025 quarterly totals
- Added data/source_dossier.xlsx and figures/build_source_data.py

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FPeEPN6oNfciD5oEqditMq
</commit_message>
<xml_diff>
--- a/data/figure_source_data.xlsx
+++ b/data/figure_source_data.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,23 +36,14 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DCE6F0"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -67,11 +58,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,16 +429,14 @@
   <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
-    <col width="42" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16" customWidth="1" style="2" min="3" max="3"/>
-    <col width="16" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16" customWidth="1" style="2" min="5" max="5"/>
-    <col width="16" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="16" customWidth="1" style="2" min="9" max="9"/>
-    <col width="16" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,27 +449,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Model: model/hf_tea_lca.py · Monte Carlo: model/monte_carlo.py → results/mc_results.npz (N = 5,000, seed 20260929)</t>
+          <t>Model: model/hf_tea_lca.py · Monte Carlo: model/monte_carlo.py -&gt; results/mc_results.npz (N = 5,000, seed 20260929) · Built by figures/build_source_data.py</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Figure</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Script</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Source of values</t>
         </is>
@@ -501,7 +488,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>– (schematic drawn by the authors)</t>
+          <t>- (schematic drawn by the authors)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -638,7 +625,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Price sources in SI Table S3; USGS MCS 2026</t>
+          <t>Price sources in SI Table S3 and the source dossier; USGS MCS 2026</t>
         </is>
       </c>
     </row>
@@ -677,7 +664,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>– (values below)</t>
+          <t>- (values below)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -707,16 +694,14 @@
   <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
-    <col width="42" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16" customWidth="1" style="2" min="3" max="3"/>
-    <col width="16" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16" customWidth="1" style="2" min="5" max="5"/>
-    <col width="16" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="16" customWidth="1" style="2" min="9" max="9"/>
-    <col width="16" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -733,6 +718,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2477,16 +2463,14 @@
   <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
-    <col width="42" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16" customWidth="1" style="2" min="3" max="3"/>
-    <col width="16" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16" customWidth="1" style="2" min="5" max="5"/>
-    <col width="16" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="16" customWidth="1" style="2" min="9" max="9"/>
-    <col width="16" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2517,16 +2501,14 @@
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
-    <col width="42" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16" customWidth="1" style="2" min="3" max="3"/>
-    <col width="16" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16" customWidth="1" style="2" min="5" max="5"/>
-    <col width="16" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="16" customWidth="1" style="2" min="9" max="9"/>
-    <col width="16" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2544,37 +2526,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Fluorspar, Technical</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>FSA, Technical</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Fluorspar, High-purity</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>FSA, High-purity</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>Fluorspar, Electronic</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>FSA, Electronic</t>
         </is>
@@ -2599,10 +2581,10 @@
         <v>0.3446</v>
       </c>
       <c r="F5" t="n">
-        <v>1.3779</v>
+        <v>1.3981</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4035</v>
+        <v>0.4094</v>
       </c>
     </row>
     <row r="6">
@@ -2612,19 +2594,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1701</v>
+        <v>0.1703</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1991</v>
+        <v>0.1993</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2331</v>
+        <v>0.2367</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -2640,19 +2622,19 @@
         <v>0.1042</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2256</v>
+        <v>0.2632</v>
       </c>
       <c r="D7" t="n">
         <v>0.1219</v>
       </c>
       <c r="E7" t="n">
-        <v>0.264</v>
+        <v>0.3079</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1427</v>
+        <v>0.1448</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3091</v>
+        <v>0.3658</v>
       </c>
     </row>
     <row r="8">
@@ -2674,10 +2656,10 @@
         <v>0.0373</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0404</v>
+        <v>0.041</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0436</v>
+        <v>0.0443</v>
       </c>
     </row>
     <row r="9">
@@ -2690,19 +2672,19 @@
         <v>0.2655</v>
       </c>
       <c r="C9" t="n">
-        <v>0.2751</v>
+        <v>0.2777</v>
       </c>
       <c r="D9" t="n">
         <v>0.3106</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3219</v>
+        <v>0.3249</v>
       </c>
       <c r="F9" t="n">
-        <v>0.3637</v>
+        <v>0.369</v>
       </c>
       <c r="G9" t="n">
-        <v>0.3769</v>
+        <v>0.386</v>
       </c>
     </row>
     <row r="10">
@@ -2724,10 +2706,10 @@
         <v>0.1516</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1776</v>
+        <v>0.1802</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1776</v>
+        <v>0.1802</v>
       </c>
     </row>
     <row r="11">
@@ -2749,7 +2731,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0379</v>
+        <v>0.0385</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -2768,10 +2750,10 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>0.4824</v>
+        <v>0.4444</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4824</v>
+        <v>0.4444</v>
       </c>
       <c r="F12" t="n">
         <v>0.9228</v>
@@ -2793,16 +2775,16 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.1805</v>
+        <v>-0.1802</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1805</v>
+        <v>-0.1802</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.3929</v>
+        <v>-0.4134</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.3929</v>
+        <v>-0.4134</v>
       </c>
     </row>
     <row r="14">
@@ -2812,48 +2794,48 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.7324</v>
+        <v>1.7325</v>
       </c>
       <c r="C14" t="n">
-        <v>0.9567</v>
+        <v>0.9969</v>
       </c>
       <c r="D14" t="n">
-        <v>2.3287</v>
+        <v>2.2912</v>
       </c>
       <c r="E14" t="n">
-        <v>1.4211</v>
+        <v>1.4305</v>
       </c>
       <c r="F14" t="n">
-        <v>2.9032</v>
+        <v>2.9176</v>
       </c>
       <c r="G14" t="n">
-        <v>1.8405</v>
+        <v>1.895</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Bracket label (per grade)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Technical</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>High-purity</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Electronic</t>
         </is>
       </c>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
+      <c r="E16" s="1" t="n"/>
+      <c r="F16" s="1" t="n"/>
+      <c r="G16" s="1" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2862,29 +2844,29 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.7756999999999999</v>
+        <v>0.7357</v>
       </c>
       <c r="C17" t="n">
-        <v>0.9076</v>
+        <v>0.8607</v>
       </c>
       <c r="D17" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ratio, fluorspar to FSA (–)</t>
+          <t>Ratio, fluorspar to FSA (-)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1.8109</v>
+        <v>1.738</v>
       </c>
       <c r="C18" t="n">
-        <v>1.6386</v>
+        <v>1.6017</v>
       </c>
       <c r="D18" t="n">
-        <v>1.5774</v>
+        <v>1.5396</v>
       </c>
     </row>
   </sheetData>
@@ -2901,16 +2883,14 @@
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
-    <col width="42" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16" customWidth="1" style="2" min="3" max="3"/>
-    <col width="16" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16" customWidth="1" style="2" min="5" max="5"/>
-    <col width="16" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="16" customWidth="1" style="2" min="9" max="9"/>
-    <col width="16" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2928,37 +2908,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Fluorspar, Technical</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>FSA, Technical</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Fluorspar, High-purity</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>FSA, High-purity</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>Fluorspar, Electronic</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>FSA, Electronic</t>
         </is>
@@ -2974,19 +2954,19 @@
         <v>0.2006</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3656</v>
+        <v>0.4031</v>
       </c>
       <c r="D5" t="n">
         <v>0.2006</v>
       </c>
       <c r="E5" t="n">
-        <v>0.3656</v>
+        <v>0.4031</v>
       </c>
       <c r="F5" t="n">
         <v>0.2006</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3656</v>
+        <v>0.4031</v>
       </c>
     </row>
     <row r="6">
@@ -2996,19 +2976,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4937</v>
+        <v>0.4944</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4937</v>
+        <v>0.4944</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4937</v>
+        <v>0.4944</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -3021,19 +3001,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3808</v>
+        <v>0.3793</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3808</v>
+        <v>0.3793</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3808</v>
+        <v>0.3793</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -3046,22 +3026,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1044</v>
+        <v>0.1047</v>
       </c>
       <c r="C8" t="n">
-        <v>1.1484</v>
+        <v>1.344</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1044</v>
+        <v>0.1047</v>
       </c>
       <c r="E8" t="n">
-        <v>1.1484</v>
+        <v>1.344</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1044</v>
+        <v>0.1047</v>
       </c>
       <c r="G8" t="n">
-        <v>1.1484</v>
+        <v>1.344</v>
       </c>
     </row>
     <row r="9">
@@ -3117,7 +3097,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Co-product credit</t>
+          <t>Purification increment</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -3127,22 +3107,22 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>0.2361</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>0.2361</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>0.5903</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>0.5903</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Purification increment</t>
+          <t>Co-product credit</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -3152,16 +3132,16 @@
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>0.2359</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>0.2359</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0.5898</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5898</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -3171,22 +3151,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.3212</v>
+        <v>1.3207</v>
       </c>
       <c r="C13" t="n">
-        <v>1.6571</v>
+        <v>1.8902</v>
       </c>
       <c r="D13" t="n">
-        <v>1.5571</v>
+        <v>1.5568</v>
       </c>
       <c r="E13" t="n">
-        <v>1.8931</v>
+        <v>2.1263</v>
       </c>
       <c r="F13" t="n">
         <v>1.911</v>
       </c>
       <c r="G13" t="n">
-        <v>2.2469</v>
+        <v>2.4805</v>
       </c>
     </row>
     <row r="14">
@@ -3199,45 +3179,45 @@
         <v>0.4722</v>
       </c>
       <c r="C14" t="n">
-        <v>0.9698</v>
+        <v>1.111</v>
       </c>
       <c r="D14" t="n">
         <v>0.6667999999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>1.1644</v>
+        <v>1.3056</v>
       </c>
       <c r="F14" t="n">
         <v>0.9587</v>
       </c>
       <c r="G14" t="n">
-        <v>1.4563</v>
+        <v>1.5975</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Bracket label (per grade)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Technical</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>High-purity</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Electronic</t>
         </is>
       </c>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
+      <c r="E16" s="1" t="n"/>
+      <c r="F16" s="1" t="n"/>
+      <c r="G16" s="1" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3246,29 +3226,29 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.3359</v>
+        <v>-0.5694</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.3359</v>
+        <v>-0.5694</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.3359</v>
+        <v>-0.5694</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ratio, fluorspar to FSA (–)</t>
+          <t>Ratio, fluorspar to FSA (-)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.7973</v>
+        <v>0.6987</v>
       </c>
       <c r="C18" t="n">
-        <v>0.8225</v>
+        <v>0.7322</v>
       </c>
       <c r="D18" t="n">
-        <v>0.8505</v>
+        <v>0.7704</v>
       </c>
     </row>
   </sheetData>
@@ -3285,16 +3265,14 @@
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
-    <col width="42" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16" customWidth="1" style="2" min="3" max="3"/>
-    <col width="16" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16" customWidth="1" style="2" min="5" max="5"/>
-    <col width="16" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="16" customWidth="1" style="2" min="9" max="9"/>
-    <col width="16" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3312,37 +3290,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Panel</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>ΔGHG at 0%</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>ΔGHG at 100%</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Break-even share (%)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3360,13 +3338,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.157</v>
+        <v>0.2661</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.7148</v>
+        <v>-0.6232</v>
       </c>
       <c r="E5" t="n">
-        <v>18</v>
+        <v>29.9</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -3391,13 +3369,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.157</v>
+        <v>0.2661</v>
       </c>
       <c r="D6" t="n">
-        <v>-1.0886</v>
+        <v>-0.997</v>
       </c>
       <c r="E6" t="n">
-        <v>12.6</v>
+        <v>21.1</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -3422,13 +3400,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.157</v>
+        <v>0.2661</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.1935</v>
+        <v>-0.0844</v>
       </c>
       <c r="E7" t="n">
-        <v>44.8</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -3453,13 +3431,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.157</v>
+        <v>0.2661</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.4505</v>
+        <v>-0.3414</v>
       </c>
       <c r="E8" t="n">
-        <v>25.8</v>
+        <v>43.8</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -3473,37 +3451,37 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>Panel</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>Low (Mt HF/yr)</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>High (Mt HF/yr)</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Fluorspar avoided low (Mt/yr)</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>Fluorspar avoided high (Mt/yr)</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3563,7 +3541,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>MarketsandMarkets 2025–2030 market value growth 6.0%/yr extended to 2035 as a volume proxy (SI Section S15); 2.14 t fluorspar/t HF</t>
+          <t>MarketsandMarkets 2025–2030 value growth 6.0%/yr extended to 2035 (SI Section S15); 2.14 t fluorspar/t HF</t>
         </is>
       </c>
     </row>
@@ -3575,24 +3553,24 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Current FSA recovery, world</t>
+          <t>Current FSA recovery, world (HF supplied)</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.3</v>
+        <v>0.232</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>0.774</v>
       </c>
       <c r="E13" t="n">
-        <v>0.642</v>
+        <v>0.497</v>
       </c>
       <c r="F13" t="n">
-        <v>2.14</v>
+        <v>1.657</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>SI Section S15; 2.14 t fluorspar/t HF</t>
+          <t>0.3–1.0 Mt HF-eq, order-of-magnitude estimate (SI Section S15); 2.14 t fluorspar/t HF</t>
         </is>
       </c>
     </row>
@@ -3604,59 +3582,59 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Potential FSA recovery</t>
+          <t>Potential FSA recovery (HF supplied)</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.5</v>
+        <v>0.387</v>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>1.549</v>
       </c>
       <c r="E14" t="n">
-        <v>1.07</v>
+        <v>0.829</v>
       </c>
       <c r="F14" t="n">
-        <v>4.28</v>
+        <v>3.315</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>SI Section S15; 2.14 t fluorspar/t HF</t>
+          <t>0.5–2.0 Mt HF-eq, order-of-magnitude estimate (SI Section S15); 2.14 t fluorspar/t HF</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Panel</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Commodity</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>China %</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>Second</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Third</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>HHI (lower bound)</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -3742,16 +3720,14 @@
   <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
-    <col width="42" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16" customWidth="1" style="2" min="3" max="3"/>
-    <col width="16" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16" customWidth="1" style="2" min="5" max="5"/>
-    <col width="16" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="16" customWidth="1" style="2" min="9" max="9"/>
-    <col width="16" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3764,42 +3740,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Base electronic-grade cost gap = 1.0627 $/kg HF; panel (a) plots the 12 inputs with the largest swing</t>
+          <t>Base electronic-grade cost gap = 1.0226 $/kg HF; panel (a) plots (gap − base)/base × 100 for the 12 inputs with the largest swing</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Panel</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Input (figure label)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Low, base, high (figure label)</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Low, base, high</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Gap at low value ($/kg HF)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Gap at high value ($/kg HF)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>Swing</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>Plotted in Fig. 4a</t>
         </is>
@@ -3818,17 +3794,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.965, 1.0, 1.84</t>
+          <t>0.956, 1.0, 1.84</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.0759</v>
+        <v>1.0396</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7462</v>
+        <v>0.6983</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3166</v>
+        <v>0.3242</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -3853,13 +3829,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.9592000000000001</v>
+        <v>0.9174</v>
       </c>
       <c r="E6" t="n">
-        <v>1.3031</v>
+        <v>1.2667</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2403</v>
+        <v>0.2441</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3875,22 +3851,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FSA price</t>
+          <t>Fluorspar price</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>93, 190, 246 $/t</t>
+          <t>405, 470, 504 $/t</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.2749</v>
+        <v>0.8292</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9403</v>
+        <v>1.1237</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2121</v>
+        <v>0.1933</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -3906,22 +3882,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Fluorspar price</t>
+          <t>FSA price</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>405, 470, 504 $/t</t>
+          <t>105, 190, 246 $/t</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.8722</v>
+        <v>1.2112</v>
       </c>
       <c r="E8" t="n">
-        <v>1.1624</v>
+        <v>0.8983</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1906</v>
+        <v>0.1886</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -3942,17 +3918,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.14, 1.37, 1.37 t/t</t>
+          <t>1.14, 1.39, 1.39 t/t</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.8815</v>
+        <v>0.836</v>
       </c>
       <c r="E9" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1812</v>
+        <v>0.1866</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -3977,13 +3953,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.925</v>
+        <v>0.8828</v>
       </c>
       <c r="E10" t="n">
-        <v>1.0824</v>
+        <v>1.0426</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1377</v>
+        <v>0.1397</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -4008,13 +3984,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1.0215</v>
+        <v>0.9807</v>
       </c>
       <c r="E11" t="n">
-        <v>1.1878</v>
+        <v>1.1494</v>
       </c>
       <c r="F11" t="n">
-        <v>0.125</v>
+        <v>0.1268</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -4039,13 +4015,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1.0546</v>
+        <v>1.0141</v>
       </c>
       <c r="E12" t="n">
-        <v>1.1764</v>
+        <v>1.141</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1137</v>
+        <v>0.1184</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -4061,22 +4037,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FSA-route steam</t>
+          <t>Steam price</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12, 12, 16 GJ/t</t>
+          <t>12.8, 18.8, 23.5 $/GJ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1.0627</v>
+        <v>1.1298</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9597</v>
+        <v>0.9382</v>
       </c>
       <c r="F13" t="n">
-        <v>0.103</v>
+        <v>0.1072</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -4101,13 +4077,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="E14" t="n">
-        <v>0.97</v>
+        <v>0.9281</v>
       </c>
       <c r="F14" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.0945</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -4123,22 +4099,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Steam price</t>
+          <t>FSA-route steam</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>12.8, 18.8, 23.5 $/GJ</t>
+          <t>12, 14, 16 GJ/t</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.152</v>
+        <v>1.0748</v>
       </c>
       <c r="E15" t="n">
-        <v>0.9925</v>
+        <v>0.9703000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0893</v>
+        <v>0.0523</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -4163,13 +4139,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1.0466</v>
+        <v>1.0062</v>
       </c>
       <c r="E16" t="n">
-        <v>1.1122</v>
+        <v>1.0728</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0495</v>
+        <v>0.0502</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -4194,13 +4170,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1.0399</v>
+        <v>0.9994</v>
       </c>
       <c r="E17" t="n">
-        <v>1.1039</v>
+        <v>1.0644</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0412</v>
+        <v>0.0418</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -4216,22 +4192,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FSA-route capital cost</t>
+          <t>Natural gas price</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2,254, 2,315, 2,466 $/(t/yr)</t>
+          <t>14.3, 16.7, 20.2 $/GJ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1.0727</v>
+        <v>1.006</v>
       </c>
       <c r="E18" t="n">
-        <v>1.0382</v>
+        <v>1.0469</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0246</v>
+        <v>0.0243</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -4247,22 +4223,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Natural gas price</t>
+          <t>FSA-route capital cost</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14.3, 16.7, 20.2 $/GJ</t>
+          <t>2,254, 2,337, 2,466 $/(t/yr)</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1.0464</v>
+        <v>1.0363</v>
       </c>
       <c r="E19" t="n">
-        <v>1.0867</v>
+        <v>1.0013</v>
       </c>
       <c r="F19" t="n">
-        <v>0.024</v>
+        <v>0.0213</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -4287,13 +4263,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.0708</v>
+        <v>1.0308</v>
       </c>
       <c r="E20" t="n">
-        <v>1.0555</v>
+        <v>1.0152</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0081</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -4318,13 +4294,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="E21" t="n">
-        <v>1.0604</v>
+        <v>1.0196</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0023</v>
+        <v>0.003</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -4349,10 +4325,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1.063</v>
+        <v>1.0229</v>
       </c>
       <c r="E22" t="n">
-        <v>1.0625</v>
+        <v>1.0223</v>
       </c>
       <c r="F22" t="n">
         <v>0.0003</v>
@@ -4371,19 +4347,19 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Labor cost</t>
+          <t>AHF plant staffing</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>20.8, 58.7, 64.0 k$/person</t>
+          <t>1.44, 1.92, 2.40 persons/kt</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="E23" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -4402,19 +4378,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AHF plant staffing</t>
+          <t>Purification capital cost</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.44, 1.92, 2.40 persons/kt</t>
+          <t>3,416, 4,764, 6,612 $/(t/yr)</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="E24" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -4433,19 +4409,19 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Purification capital cost</t>
+          <t>Industrial-grade HF price</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>3,416, 4,764, 6,612 $/(t/yr)</t>
+          <t>787, 1,060, 1,600 $/t</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="E25" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -4464,19 +4440,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Industrial-grade HF price</t>
+          <t>Labor cost</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>788, 1,062, 1,602 $/t</t>
+          <t>20.8, 58.7, 64.0 k$/person</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="E26" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -4504,10 +4480,10 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="E27" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -4535,10 +4511,10 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="E28" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -4566,10 +4542,10 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="E29" t="n">
-        <v>1.0627</v>
+        <v>1.0226</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -4581,37 +4557,37 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>Panel</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>Grade</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>Median</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>P95</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>Share of draws with gap &gt; 0</t>
         </is>
       </c>
-      <c r="G31" s="3" t="n"/>
+      <c r="G31" s="1" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4625,13 +4601,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.5477</v>
+        <v>0.5312</v>
       </c>
       <c r="D32" t="n">
-        <v>0.7374000000000001</v>
+        <v>0.7198</v>
       </c>
       <c r="E32" t="n">
-        <v>0.9403</v>
+        <v>0.9197</v>
       </c>
       <c r="F32" t="n">
         <v>1</v>
@@ -4649,13 +4625,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.6313</v>
+        <v>0.6114000000000001</v>
       </c>
       <c r="D33" t="n">
-        <v>0.8548</v>
+        <v>0.8348</v>
       </c>
       <c r="E33" t="n">
-        <v>1.0992</v>
+        <v>1.0758</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
@@ -4673,13 +4649,13 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.6303</v>
+        <v>0.617</v>
       </c>
       <c r="D34" t="n">
-        <v>0.8988</v>
+        <v>0.8855</v>
       </c>
       <c r="E34" t="n">
-        <v>1.1785</v>
+        <v>1.1673</v>
       </c>
       <c r="F34" t="n">
         <v>1</v>
@@ -4699,16 +4675,14 @@
   <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
-    <col width="42" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16" customWidth="1" style="2" min="3" max="3"/>
-    <col width="16" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16" customWidth="1" style="2" min="5" max="5"/>
-    <col width="16" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="16" customWidth="1" style="2" min="9" max="9"/>
-    <col width="16" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4721,47 +4695,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cost gap 1.0627 $/kg HF (= $ million per kt); MC 5–95% 0.6303–1.1785; upper axis = volume / 350 kt/yr</t>
+          <t>Cost gap 1.0226 $/kg HF (= $ million per kt); Monte Carlo 5–95% 0.6170–1.1673; world electronic-grade demand 350 kt/yr for the upper axis</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Annual volume (kt/yr)</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Share of demand at 350 kt/yr (%)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>1.5 yr</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>3 yr</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>5 yr</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>10 yr</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>5 yr, P5 gap</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>5 yr, P95 gap</t>
         </is>
@@ -4801,22 +4775,22 @@
         <v>0.143</v>
       </c>
       <c r="C6" t="n">
-        <v>0.797</v>
+        <v>0.767</v>
       </c>
       <c r="D6" t="n">
-        <v>1.594</v>
+        <v>1.534</v>
       </c>
       <c r="E6" t="n">
-        <v>2.657</v>
+        <v>2.556</v>
       </c>
       <c r="F6" t="n">
-        <v>5.314</v>
+        <v>5.113</v>
       </c>
       <c r="G6" t="n">
-        <v>1.576</v>
+        <v>1.543</v>
       </c>
       <c r="H6" t="n">
-        <v>2.946</v>
+        <v>2.918</v>
       </c>
     </row>
     <row r="7">
@@ -4827,22 +4801,22 @@
         <v>0.286</v>
       </c>
       <c r="C7" t="n">
-        <v>1.594</v>
+        <v>1.534</v>
       </c>
       <c r="D7" t="n">
-        <v>3.188</v>
+        <v>3.068</v>
       </c>
       <c r="E7" t="n">
-        <v>5.314</v>
+        <v>5.113</v>
       </c>
       <c r="F7" t="n">
-        <v>10.627</v>
+        <v>10.226</v>
       </c>
       <c r="G7" t="n">
-        <v>3.151</v>
+        <v>3.085</v>
       </c>
       <c r="H7" t="n">
-        <v>5.892</v>
+        <v>5.836</v>
       </c>
     </row>
     <row r="8">
@@ -4853,22 +4827,22 @@
         <v>0.429</v>
       </c>
       <c r="C8" t="n">
-        <v>2.391</v>
+        <v>2.301</v>
       </c>
       <c r="D8" t="n">
-        <v>4.782</v>
+        <v>4.602</v>
       </c>
       <c r="E8" t="n">
-        <v>7.971</v>
+        <v>7.669</v>
       </c>
       <c r="F8" t="n">
-        <v>15.941</v>
+        <v>15.339</v>
       </c>
       <c r="G8" t="n">
-        <v>4.727</v>
+        <v>4.628</v>
       </c>
       <c r="H8" t="n">
-        <v>8.837999999999999</v>
+        <v>8.755000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -4879,22 +4853,22 @@
         <v>0.571</v>
       </c>
       <c r="C9" t="n">
-        <v>3.188</v>
+        <v>3.068</v>
       </c>
       <c r="D9" t="n">
-        <v>6.376</v>
+        <v>6.135</v>
       </c>
       <c r="E9" t="n">
-        <v>10.627</v>
+        <v>10.226</v>
       </c>
       <c r="F9" t="n">
-        <v>21.255</v>
+        <v>20.452</v>
       </c>
       <c r="G9" t="n">
-        <v>6.303</v>
+        <v>6.17</v>
       </c>
       <c r="H9" t="n">
-        <v>11.785</v>
+        <v>11.673</v>
       </c>
     </row>
     <row r="10">
@@ -4905,22 +4879,22 @@
         <v>0.714</v>
       </c>
       <c r="C10" t="n">
-        <v>3.985</v>
+        <v>3.835</v>
       </c>
       <c r="D10" t="n">
-        <v>7.971</v>
+        <v>7.669</v>
       </c>
       <c r="E10" t="n">
-        <v>13.284</v>
+        <v>12.782</v>
       </c>
       <c r="F10" t="n">
-        <v>26.569</v>
+        <v>25.564</v>
       </c>
       <c r="G10" t="n">
-        <v>7.878</v>
+        <v>7.713</v>
       </c>
       <c r="H10" t="n">
-        <v>14.731</v>
+        <v>14.591</v>
       </c>
     </row>
     <row r="11">
@@ -4931,22 +4905,22 @@
         <v>0.857</v>
       </c>
       <c r="C11" t="n">
-        <v>4.782</v>
+        <v>4.602</v>
       </c>
       <c r="D11" t="n">
-        <v>9.565</v>
+        <v>9.202999999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>15.941</v>
+        <v>15.339</v>
       </c>
       <c r="F11" t="n">
-        <v>31.882</v>
+        <v>30.677</v>
       </c>
       <c r="G11" t="n">
-        <v>9.454000000000001</v>
+        <v>9.255000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>17.677</v>
+        <v>17.509</v>
       </c>
     </row>
     <row r="12">
@@ -4957,22 +4931,22 @@
         <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>5.579</v>
+        <v>5.369</v>
       </c>
       <c r="D12" t="n">
-        <v>11.159</v>
+        <v>10.737</v>
       </c>
       <c r="E12" t="n">
-        <v>18.598</v>
+        <v>17.895</v>
       </c>
       <c r="F12" t="n">
-        <v>37.196</v>
+        <v>35.79</v>
       </c>
       <c r="G12" t="n">
-        <v>11.03</v>
+        <v>10.798</v>
       </c>
       <c r="H12" t="n">
-        <v>20.623</v>
+        <v>20.427</v>
       </c>
     </row>
     <row r="13">
@@ -4983,22 +4957,22 @@
         <v>1.143</v>
       </c>
       <c r="C13" t="n">
-        <v>6.376</v>
+        <v>6.135</v>
       </c>
       <c r="D13" t="n">
-        <v>12.753</v>
+        <v>12.271</v>
       </c>
       <c r="E13" t="n">
-        <v>21.255</v>
+        <v>20.452</v>
       </c>
       <c r="F13" t="n">
-        <v>42.51</v>
+        <v>40.903</v>
       </c>
       <c r="G13" t="n">
-        <v>12.605</v>
+        <v>12.34</v>
       </c>
       <c r="H13" t="n">
-        <v>23.569</v>
+        <v>23.345</v>
       </c>
     </row>
     <row r="14">
@@ -5009,22 +4983,22 @@
         <v>1.286</v>
       </c>
       <c r="C14" t="n">
-        <v>7.174</v>
+        <v>6.902</v>
       </c>
       <c r="D14" t="n">
-        <v>14.347</v>
+        <v>13.805</v>
       </c>
       <c r="E14" t="n">
-        <v>23.912</v>
+        <v>23.008</v>
       </c>
       <c r="F14" t="n">
-        <v>47.824</v>
+        <v>46.016</v>
       </c>
       <c r="G14" t="n">
-        <v>14.181</v>
+        <v>13.883</v>
       </c>
       <c r="H14" t="n">
-        <v>26.515</v>
+        <v>26.264</v>
       </c>
     </row>
     <row r="15">
@@ -5035,22 +5009,22 @@
         <v>1.429</v>
       </c>
       <c r="C15" t="n">
-        <v>7.971</v>
+        <v>7.669</v>
       </c>
       <c r="D15" t="n">
-        <v>15.941</v>
+        <v>15.339</v>
       </c>
       <c r="E15" t="n">
-        <v>26.569</v>
+        <v>25.564</v>
       </c>
       <c r="F15" t="n">
-        <v>53.137</v>
+        <v>51.129</v>
       </c>
       <c r="G15" t="n">
-        <v>15.757</v>
+        <v>15.426</v>
       </c>
       <c r="H15" t="n">
-        <v>29.461</v>
+        <v>29.182</v>
       </c>
     </row>
     <row r="16">
@@ -5061,22 +5035,22 @@
         <v>1.571</v>
       </c>
       <c r="C16" t="n">
-        <v>8.768000000000001</v>
+        <v>8.436</v>
       </c>
       <c r="D16" t="n">
-        <v>17.535</v>
+        <v>16.873</v>
       </c>
       <c r="E16" t="n">
-        <v>29.226</v>
+        <v>28.121</v>
       </c>
       <c r="F16" t="n">
-        <v>58.451</v>
+        <v>56.242</v>
       </c>
       <c r="G16" t="n">
-        <v>17.332</v>
+        <v>16.968</v>
       </c>
       <c r="H16" t="n">
-        <v>32.408</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="17">
@@ -5087,22 +5061,22 @@
         <v>1.714</v>
       </c>
       <c r="C17" t="n">
-        <v>9.565</v>
+        <v>9.202999999999999</v>
       </c>
       <c r="D17" t="n">
-        <v>19.129</v>
+        <v>18.406</v>
       </c>
       <c r="E17" t="n">
-        <v>31.882</v>
+        <v>30.677</v>
       </c>
       <c r="F17" t="n">
-        <v>63.765</v>
+        <v>61.355</v>
       </c>
       <c r="G17" t="n">
-        <v>18.908</v>
+        <v>18.511</v>
       </c>
       <c r="H17" t="n">
-        <v>35.354</v>
+        <v>35.018</v>
       </c>
     </row>
     <row r="18">
@@ -5113,22 +5087,22 @@
         <v>1.857</v>
       </c>
       <c r="C18" t="n">
-        <v>10.362</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="D18" t="n">
-        <v>20.724</v>
+        <v>19.94</v>
       </c>
       <c r="E18" t="n">
-        <v>34.539</v>
+        <v>33.234</v>
       </c>
       <c r="F18" t="n">
-        <v>69.078</v>
+        <v>66.468</v>
       </c>
       <c r="G18" t="n">
-        <v>20.484</v>
+        <v>20.053</v>
       </c>
       <c r="H18" t="n">
-        <v>38.3</v>
+        <v>37.936</v>
       </c>
     </row>
     <row r="19">
@@ -5139,22 +5113,22 @@
         <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>11.159</v>
+        <v>10.737</v>
       </c>
       <c r="D19" t="n">
-        <v>22.318</v>
+        <v>21.474</v>
       </c>
       <c r="E19" t="n">
-        <v>37.196</v>
+        <v>35.79</v>
       </c>
       <c r="F19" t="n">
-        <v>74.392</v>
+        <v>71.581</v>
       </c>
       <c r="G19" t="n">
-        <v>22.059</v>
+        <v>21.596</v>
       </c>
       <c r="H19" t="n">
-        <v>41.246</v>
+        <v>40.854</v>
       </c>
     </row>
     <row r="20">
@@ -5165,22 +5139,22 @@
         <v>2.143</v>
       </c>
       <c r="C20" t="n">
-        <v>11.956</v>
+        <v>11.504</v>
       </c>
       <c r="D20" t="n">
-        <v>23.912</v>
+        <v>23.008</v>
       </c>
       <c r="E20" t="n">
-        <v>39.853</v>
+        <v>38.347</v>
       </c>
       <c r="F20" t="n">
-        <v>79.706</v>
+        <v>76.693</v>
       </c>
       <c r="G20" t="n">
-        <v>23.635</v>
+        <v>23.138</v>
       </c>
       <c r="H20" t="n">
-        <v>44.192</v>
+        <v>43.773</v>
       </c>
     </row>
     <row r="21">
@@ -5191,49 +5165,49 @@
         <v>2.286</v>
       </c>
       <c r="C21" t="n">
-        <v>12.753</v>
+        <v>12.271</v>
       </c>
       <c r="D21" t="n">
-        <v>25.506</v>
+        <v>24.542</v>
       </c>
       <c r="E21" t="n">
-        <v>42.51</v>
+        <v>40.903</v>
       </c>
       <c r="F21" t="n">
-        <v>85.02</v>
+        <v>81.806</v>
       </c>
       <c r="G21" t="n">
-        <v>25.211</v>
+        <v>24.681</v>
       </c>
       <c r="H21" t="n">
-        <v>47.138</v>
+        <v>46.691</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>Marker</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Volume (kt/yr)</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>Share of demand (%)</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Calculation</t>
         </is>
       </c>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
+      <c r="E23" s="1" t="n"/>
+      <c r="F23" s="1" t="n"/>
+      <c r="G23" s="1" t="n"/>
+      <c r="H23" s="1" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5242,11 +5216,11 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1.882</v>
+        <v>1.956</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.47–0.63</t>
+          <t>0.49–0.65</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -5262,11 +5236,11 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>6.273</v>
+        <v>6.519</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1.57–2.09</t>
+          <t>1.63–2.17</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -5282,11 +5256,11 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3.173</v>
+        <v>3.241</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>0.79–1.06</t>
+          <t>0.81–1.08</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5309,16 +5283,14 @@
   <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
-    <col width="42" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16" customWidth="1" style="2" min="3" max="3"/>
-    <col width="16" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16" customWidth="1" style="2" min="5" max="5"/>
-    <col width="16" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="16" customWidth="1" style="2" min="9" max="9"/>
-    <col width="16" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5335,53 +5307,54 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Panel</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Grade</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Series</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Marker</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Plotted value</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
@@ -5663,41 +5636,38 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Panel</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Share of world (%)</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5881,16 +5851,14 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="2" min="1" max="1"/>
-    <col width="42" customWidth="1" style="2" min="2" max="2"/>
-    <col width="16" customWidth="1" style="2" min="3" max="3"/>
-    <col width="16" customWidth="1" style="2" min="4" max="4"/>
-    <col width="16" customWidth="1" style="2" min="5" max="5"/>
-    <col width="16" customWidth="1" style="2" min="6" max="6"/>
-    <col width="16" customWidth="1" style="2" min="7" max="7"/>
-    <col width="16" customWidth="1" style="2" min="8" max="8"/>
-    <col width="16" customWidth="1" style="2" min="9" max="9"/>
-    <col width="16" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5908,27 +5876,27 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Flow</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Base method</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Base value</t>
         </is>
@@ -5957,7 +5925,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.37 kg CO2eq/kg HF</t>
+          <t>0.40 kg CO2eq/kg HF</t>
         </is>
       </c>
     </row>
@@ -6065,7 +6033,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.73% of burden</t>
+          <t>0.82% of burden</t>
         </is>
       </c>
     </row>

</xml_diff>